<commit_message>
feat: release Hall data 20260912-v001
</commit_message>
<xml_diff>
--- a/data/checkmate/hall_fame.xlsx
+++ b/data/checkmate/hall_fame.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\projects_2027\checkee_2026\data\checkmate\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B919C7E5-BBFD-4D21-AB8C-49043C4F287F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{847635D8-6011-421A-B7DD-8B262319D0CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="7380" yWindow="4000" windowWidth="28800" windowHeight="15370" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="6980" yWindow="5440" windowWidth="28800" windowHeight="15370" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="845" uniqueCount="283">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="842" uniqueCount="284">
   <si>
     <t>地点</t>
   </si>
@@ -375,9 +375,6 @@
     <t>ufun-checkee-044</t>
   </si>
   <si>
-    <t>uci</t>
-  </si>
-  <si>
     <t>ufun-checkee-045</t>
   </si>
   <si>
@@ -433,9 +430,6 @@
   </si>
   <si>
     <t>ufun-checkee-055</t>
-  </si>
-  <si>
-    <t>ufun-checkee-056</t>
   </si>
   <si>
     <t>Phy</t>
@@ -1162,6 +1156,17 @@
   </si>
   <si>
     <t>ES</t>
+    <phoneticPr fontId="13" type="noConversion"/>
+  </si>
+  <si>
+    <t>ufun-checkee-115</t>
+  </si>
+  <si>
+    <t>JMY</t>
+    <phoneticPr fontId="13" type="noConversion"/>
+  </si>
+  <si>
+    <t>金牌狗啃包</t>
     <phoneticPr fontId="13" type="noConversion"/>
   </si>
 </sst>
@@ -1369,7 +1374,7 @@
     <xf numFmtId="0" fontId="0" fillId="6" borderId="2"/>
     <xf numFmtId="0" fontId="12" fillId="6" borderId="2"/>
   </cellStyleXfs>
-  <cellXfs count="58">
+  <cellXfs count="55">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -1526,16 +1531,7 @@
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="2" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1751,7 +1747,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:S194"/>
+  <dimension ref="A1:S193"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="14.83203125" style="37" customWidth="1"/>
@@ -1767,7 +1763,7 @@
   <sheetData>
     <row r="1" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A1" s="41" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>0</v>
@@ -1800,7 +1796,7 @@
         <v>8</v>
       </c>
       <c r="L1" s="43" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="M1" s="6"/>
       <c r="N1" s="6"/>
@@ -1814,7 +1810,7 @@
     </row>
     <row r="2" spans="1:19" s="37" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A2" s="45" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="B2" s="6" t="s">
         <v>10</v>
@@ -1851,7 +1847,7 @@
     </row>
     <row r="3" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A3" s="41" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="B3" s="6" t="s">
         <v>10</v>
@@ -1860,7 +1856,7 @@
         <v>16</v>
       </c>
       <c r="D3" s="34" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="E3" s="38" t="s">
         <v>13</v>
@@ -1873,10 +1869,10 @@
       </c>
       <c r="H3" s="12"/>
       <c r="I3" s="34" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="J3" s="34" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="K3" s="6"/>
       <c r="L3" s="6"/>
@@ -1892,7 +1888,7 @@
     </row>
     <row r="4" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A4" s="45" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="B4" s="6" t="s">
         <v>10</v>
@@ -1931,7 +1927,7 @@
     </row>
     <row r="5" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A5" s="45" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="B5" s="6" t="s">
         <v>10</v>
@@ -1940,7 +1936,7 @@
         <v>16</v>
       </c>
       <c r="D5" s="34" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="E5" s="7" t="s">
         <v>17</v>
@@ -1953,10 +1949,10 @@
       </c>
       <c r="H5" s="13"/>
       <c r="I5" s="34" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="J5" s="34" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="K5" s="6"/>
       <c r="L5" s="6"/>
@@ -1972,7 +1968,7 @@
     </row>
     <row r="6" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A6" s="41" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="B6" s="6" t="s">
         <v>20</v>
@@ -1993,7 +1989,7 @@
         <v>14</v>
       </c>
       <c r="H6" s="12"/>
-      <c r="I6" s="6"/>
+      <c r="I6" s="34"/>
       <c r="J6" s="6"/>
       <c r="K6" s="6"/>
       <c r="L6" s="6"/>
@@ -2008,13 +2004,18 @@
       </c>
     </row>
     <row r="7" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="A7" s="41" t="s">
+        <v>282</v>
+      </c>
       <c r="B7" s="6" t="s">
         <v>10</v>
       </c>
       <c r="C7" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="D7" s="7"/>
+      <c r="D7" s="34" t="s">
+        <v>242</v>
+      </c>
       <c r="E7" s="7" t="s">
         <v>17</v>
       </c>
@@ -2025,7 +2026,9 @@
         <v>14</v>
       </c>
       <c r="H7" s="12"/>
-      <c r="I7" s="6"/>
+      <c r="I7" s="34" t="s">
+        <v>227</v>
+      </c>
       <c r="J7" s="6"/>
       <c r="K7" s="6"/>
       <c r="L7" s="6"/>
@@ -2041,7 +2044,7 @@
     </row>
     <row r="8" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A8" s="41" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="B8" s="6" t="s">
         <v>10</v>
@@ -2082,7 +2085,7 @@
     </row>
     <row r="9" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A9" s="41" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="B9" s="6" t="s">
         <v>10</v>
@@ -2104,7 +2107,7 @@
       </c>
       <c r="H9" s="12"/>
       <c r="I9" s="34" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="J9" s="6"/>
       <c r="K9" s="6"/>
@@ -2161,7 +2164,7 @@
     </row>
     <row r="11" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A11" s="45" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="B11" s="6" t="s">
         <v>10</v>
@@ -2170,7 +2173,7 @@
         <v>11</v>
       </c>
       <c r="D11" s="34" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="E11" s="42" t="s">
         <v>28</v>
@@ -2183,7 +2186,7 @@
       </c>
       <c r="H11" s="12"/>
       <c r="I11" s="34" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="J11" s="6"/>
       <c r="K11" s="6"/>
@@ -2340,7 +2343,7 @@
     </row>
     <row r="16" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A16" s="41" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="B16" s="6" t="s">
         <v>20</v>
@@ -2349,7 +2352,7 @@
         <v>11</v>
       </c>
       <c r="D16" s="34" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="E16" s="7" t="s">
         <v>28</v>
@@ -2362,7 +2365,7 @@
       </c>
       <c r="H16" s="12"/>
       <c r="I16" s="34" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="J16" s="34"/>
       <c r="K16" s="6"/>
@@ -2385,10 +2388,10 @@
         <v>11</v>
       </c>
       <c r="D17" s="34" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="E17" s="7" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="F17" s="8">
         <v>46154</v>
@@ -2398,10 +2401,10 @@
       </c>
       <c r="H17" s="12"/>
       <c r="I17" s="34" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="J17" s="34" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="K17" s="6"/>
       <c r="L17" s="6"/>
@@ -2529,7 +2532,7 @@
     </row>
     <row r="21" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A21" s="45" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="B21" s="6" t="s">
         <v>10</v>
@@ -2551,7 +2554,7 @@
       </c>
       <c r="H21" s="12"/>
       <c r="I21" s="34" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="J21" s="6" t="s">
         <v>43</v>
@@ -2570,7 +2573,7 @@
     </row>
     <row r="22" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A22" s="45" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="B22" s="6" t="s">
         <v>20</v>
@@ -2579,7 +2582,7 @@
         <v>11</v>
       </c>
       <c r="D22" s="34" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="E22" s="7" t="s">
         <v>28</v>
@@ -2592,10 +2595,10 @@
       </c>
       <c r="H22" s="13"/>
       <c r="I22" s="34" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="J22" s="34" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="K22" s="6"/>
       <c r="L22" s="6"/>
@@ -2649,7 +2652,7 @@
     </row>
     <row r="24" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A24" s="41" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="B24" s="6" t="s">
         <v>10</v>
@@ -2658,7 +2661,7 @@
         <v>11</v>
       </c>
       <c r="D24" s="34" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="E24" s="7" t="s">
         <v>28</v>
@@ -2671,11 +2674,11 @@
       </c>
       <c r="H24" s="12"/>
       <c r="I24" s="34" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="J24" s="6"/>
       <c r="K24" s="34" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="L24" s="6"/>
       <c r="M24" s="6"/>
@@ -3053,6 +3056,9 @@
       </c>
     </row>
     <row r="35" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="A35" s="45" t="s">
+        <v>283</v>
+      </c>
       <c r="B35" s="6" t="s">
         <v>20</v>
       </c>
@@ -3110,7 +3116,7 @@
       <c r="H36" s="12"/>
       <c r="I36" s="6"/>
       <c r="J36" s="34" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="K36" s="6" t="s">
         <v>30</v>
@@ -3162,47 +3168,47 @@
         <v>95</v>
       </c>
     </row>
-    <row r="38" spans="1:19" s="56" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:19" s="37" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A38" s="41" t="s">
-        <v>279</v>
-      </c>
-      <c r="B38" s="54" t="s">
+        <v>277</v>
+      </c>
+      <c r="B38" s="48" t="s">
         <v>20</v>
       </c>
-      <c r="C38" s="54" t="s">
+      <c r="C38" s="48" t="s">
         <v>16</v>
       </c>
       <c r="D38" s="34" t="s">
-        <v>282</v>
-      </c>
-      <c r="E38" s="55" t="s">
+        <v>280</v>
+      </c>
+      <c r="E38" s="9" t="s">
         <v>67</v>
       </c>
       <c r="F38" s="8">
         <v>46181</v>
       </c>
-      <c r="G38" s="55" t="s">
+      <c r="G38" s="9" t="s">
         <v>14</v>
       </c>
       <c r="H38" s="12"/>
-      <c r="I38" s="57" t="s">
-        <v>239</v>
-      </c>
-      <c r="J38" s="57" t="s">
-        <v>280</v>
-      </c>
-      <c r="K38" s="57" t="s">
+      <c r="I38" s="54" t="s">
+        <v>237</v>
+      </c>
+      <c r="J38" s="54" t="s">
+        <v>278</v>
+      </c>
+      <c r="K38" s="54" t="s">
+        <v>279</v>
+      </c>
+      <c r="L38" s="48"/>
+      <c r="M38" s="48"/>
+      <c r="N38" s="48"/>
+      <c r="O38" s="48"/>
+      <c r="P38" s="48"/>
+      <c r="Q38" s="48"/>
+      <c r="R38" s="48"/>
+      <c r="S38" t="s">
         <v>281</v>
-      </c>
-      <c r="L38" s="54"/>
-      <c r="M38" s="54"/>
-      <c r="N38" s="54"/>
-      <c r="O38" s="54"/>
-      <c r="P38" s="54"/>
-      <c r="Q38" s="54"/>
-      <c r="R38" s="54"/>
-      <c r="S38" t="str">
-        <v>ufun-checkee-115</v>
       </c>
     </row>
     <row r="39" spans="1:19" x14ac:dyDescent="0.35">
@@ -3213,7 +3219,7 @@
         <v>16</v>
       </c>
       <c r="D39" s="34" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="E39" s="7" t="s">
         <v>67</v>
@@ -3497,7 +3503,7 @@
     </row>
     <row r="47" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A47" s="45" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="B47" s="6" t="s">
         <v>20</v>
@@ -3506,7 +3512,7 @@
         <v>16</v>
       </c>
       <c r="D47" s="34" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="E47" s="7" t="s">
         <v>67</v>
@@ -3519,10 +3525,10 @@
       </c>
       <c r="H47" s="12"/>
       <c r="I47" s="34" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="J47" s="34" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="K47" s="6"/>
       <c r="L47" s="6"/>
@@ -3533,12 +3539,12 @@
       <c r="Q47" s="6"/>
       <c r="R47" s="6"/>
       <c r="S47" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="48" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A48" s="41" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="B48" s="6" t="s">
         <v>10</v>
@@ -3547,7 +3553,7 @@
         <v>16</v>
       </c>
       <c r="D48" s="34" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="E48" s="7" t="s">
         <v>67</v>
@@ -3560,10 +3566,10 @@
       </c>
       <c r="H48" s="12"/>
       <c r="I48" s="34" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="J48" s="34" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="K48" s="6"/>
       <c r="L48" s="6"/>
@@ -3574,7 +3580,7 @@
       <c r="Q48" s="6"/>
       <c r="R48" s="6"/>
       <c r="S48" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="49" spans="2:19" x14ac:dyDescent="0.35">
@@ -3608,7 +3614,7 @@
       <c r="Q49" s="6"/>
       <c r="R49" s="6"/>
       <c r="S49" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="50" spans="2:19" x14ac:dyDescent="0.35">
@@ -3648,7 +3654,7 @@
       <c r="Q50" s="6"/>
       <c r="R50" s="6"/>
       <c r="S50" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="51" spans="2:19" x14ac:dyDescent="0.35">
@@ -3688,7 +3694,7 @@
       <c r="Q51" s="6"/>
       <c r="R51" s="6"/>
       <c r="S51" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="52" spans="2:19" x14ac:dyDescent="0.35">
@@ -3724,7 +3730,7 @@
       <c r="Q52" s="6"/>
       <c r="R52" s="6"/>
       <c r="S52" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="53" spans="2:19" x14ac:dyDescent="0.35">
@@ -3762,7 +3768,7 @@
       <c r="Q53" s="21"/>
       <c r="R53" s="21"/>
       <c r="S53" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="54" spans="2:19" x14ac:dyDescent="0.35">
@@ -3800,7 +3806,7 @@
       <c r="Q54" s="21"/>
       <c r="R54" s="21"/>
       <c r="S54" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="55" spans="2:19" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
@@ -3832,7 +3838,7 @@
       <c r="Q55" s="21"/>
       <c r="R55" s="21"/>
       <c r="S55" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="56" spans="2:19" x14ac:dyDescent="0.35">
@@ -3866,7 +3872,7 @@
       <c r="Q56" s="21"/>
       <c r="R56" s="21"/>
       <c r="S56" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="57" spans="2:19" x14ac:dyDescent="0.35">
@@ -3900,18 +3906,18 @@
       <c r="Q57" s="21"/>
       <c r="R57" s="21"/>
       <c r="S57" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="58" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B58" s="6" t="s">
-        <v>63</v>
+        <v>20</v>
       </c>
       <c r="C58" s="6" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="D58" s="7" t="s">
-        <v>35</v>
+        <v>21</v>
       </c>
       <c r="E58" s="7" t="s">
         <v>67</v>
@@ -3923,13 +3929,9 @@
         <v>14</v>
       </c>
       <c r="H58" s="12"/>
-      <c r="I58" s="6" t="s">
-        <v>113</v>
-      </c>
+      <c r="I58" s="6"/>
       <c r="J58" s="6"/>
-      <c r="K58" s="6" t="s">
-        <v>64</v>
-      </c>
+      <c r="K58" s="6"/>
       <c r="L58" s="21"/>
       <c r="M58" s="21"/>
       <c r="N58" s="21"/>
@@ -3943,13 +3945,13 @@
     </row>
     <row r="59" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B59" s="6" t="s">
-        <v>20</v>
+        <v>99</v>
       </c>
       <c r="C59" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="D59" s="7" t="s">
-        <v>21</v>
+      <c r="D59" s="34" t="s">
+        <v>216</v>
       </c>
       <c r="E59" s="7" t="s">
         <v>67</v>
@@ -3961,9 +3963,15 @@
         <v>14</v>
       </c>
       <c r="H59" s="12"/>
-      <c r="I59" s="6"/>
-      <c r="J59" s="6"/>
-      <c r="K59" s="6"/>
+      <c r="I59" s="15" t="s">
+        <v>115</v>
+      </c>
+      <c r="J59" s="34" t="s">
+        <v>216</v>
+      </c>
+      <c r="K59" s="34" t="s">
+        <v>215</v>
+      </c>
       <c r="L59" s="21"/>
       <c r="M59" s="21"/>
       <c r="N59" s="21"/>
@@ -3972,7 +3980,7 @@
       <c r="Q59" s="21"/>
       <c r="R59" s="21"/>
       <c r="S59" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
     </row>
     <row r="60" spans="2:19" x14ac:dyDescent="0.35">
@@ -3982,27 +3990,23 @@
       <c r="C60" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="D60" s="34" t="s">
-        <v>218</v>
-      </c>
+      <c r="D60" s="7"/>
       <c r="E60" s="7" t="s">
         <v>67</v>
       </c>
       <c r="F60" s="8">
-        <v>46189</v>
+        <v>46190</v>
       </c>
       <c r="G60" s="7" t="s">
         <v>14</v>
       </c>
       <c r="H60" s="12"/>
-      <c r="I60" s="15" t="s">
-        <v>116</v>
-      </c>
-      <c r="J60" s="34" t="s">
-        <v>218</v>
-      </c>
-      <c r="K60" s="34" t="s">
-        <v>217</v>
+      <c r="I60" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="J60" s="6"/>
+      <c r="K60" s="6" t="s">
+        <v>117</v>
       </c>
       <c r="L60" s="21"/>
       <c r="M60" s="21"/>
@@ -4017,28 +4021,30 @@
     </row>
     <row r="61" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B61" s="6" t="s">
-        <v>99</v>
+        <v>58</v>
       </c>
       <c r="C61" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="D61" s="7"/>
+        <v>11</v>
+      </c>
+      <c r="D61" s="7" t="s">
+        <v>73</v>
+      </c>
       <c r="E61" s="7" t="s">
         <v>67</v>
       </c>
       <c r="F61" s="8">
-        <v>46190</v>
+        <v>46191</v>
       </c>
       <c r="G61" s="7" t="s">
-        <v>14</v>
+        <v>68</v>
       </c>
       <c r="H61" s="12"/>
-      <c r="I61" s="6" t="s">
-        <v>104</v>
+      <c r="I61" s="21" t="s">
+        <v>115</v>
       </c>
       <c r="J61" s="6"/>
-      <c r="K61" s="6" t="s">
-        <v>118</v>
+      <c r="K61" s="35" t="s">
+        <v>119</v>
       </c>
       <c r="L61" s="21"/>
       <c r="M61" s="21"/>
@@ -4053,14 +4059,12 @@
     </row>
     <row r="62" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B62" s="6" t="s">
-        <v>58</v>
+        <v>99</v>
       </c>
       <c r="C62" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="D62" s="7" t="s">
-        <v>73</v>
-      </c>
+      <c r="D62" s="7"/>
       <c r="E62" s="7" t="s">
         <v>67</v>
       </c>
@@ -4068,15 +4072,15 @@
         <v>46191</v>
       </c>
       <c r="G62" s="7" t="s">
-        <v>68</v>
+        <v>14</v>
       </c>
       <c r="H62" s="12"/>
-      <c r="I62" s="21" t="s">
-        <v>116</v>
+      <c r="I62" s="6" t="s">
+        <v>121</v>
       </c>
       <c r="J62" s="6"/>
-      <c r="K62" s="35" t="s">
-        <v>120</v>
+      <c r="K62" s="6" t="s">
+        <v>122</v>
       </c>
       <c r="L62" s="21"/>
       <c r="M62" s="21"/>
@@ -4086,34 +4090,34 @@
       <c r="Q62" s="21"/>
       <c r="R62" s="21"/>
       <c r="S62" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
     </row>
     <row r="63" spans="2:19" x14ac:dyDescent="0.35">
-      <c r="B63" s="6" t="s">
-        <v>99</v>
-      </c>
-      <c r="C63" s="6" t="s">
+      <c r="B63" s="16" t="s">
+        <v>20</v>
+      </c>
+      <c r="C63" s="16" t="s">
         <v>11</v>
       </c>
-      <c r="D63" s="7"/>
-      <c r="E63" s="7" t="s">
+      <c r="D63" s="17" t="s">
+        <v>21</v>
+      </c>
+      <c r="E63" s="18" t="s">
         <v>67</v>
       </c>
-      <c r="F63" s="8">
+      <c r="F63" s="19">
         <v>46191</v>
       </c>
-      <c r="G63" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="H63" s="12"/>
-      <c r="I63" s="6" t="s">
-        <v>122</v>
+      <c r="G63" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="H63" s="20"/>
+      <c r="I63" s="16" t="s">
+        <v>124</v>
       </c>
       <c r="J63" s="6"/>
-      <c r="K63" s="6" t="s">
-        <v>123</v>
-      </c>
+      <c r="K63" s="6"/>
       <c r="L63" s="21"/>
       <c r="M63" s="21"/>
       <c r="N63" s="21"/>
@@ -4122,32 +4126,28 @@
       <c r="Q63" s="21"/>
       <c r="R63" s="21"/>
       <c r="S63" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="64" spans="2:19" x14ac:dyDescent="0.35">
-      <c r="B64" s="16" t="s">
-        <v>20</v>
-      </c>
-      <c r="C64" s="16" t="s">
-        <v>11</v>
-      </c>
-      <c r="D64" s="17" t="s">
-        <v>21</v>
-      </c>
-      <c r="E64" s="18" t="s">
+      <c r="B64" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="C64" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="D64" s="7"/>
+      <c r="E64" s="7" t="s">
         <v>67</v>
       </c>
-      <c r="F64" s="19">
+      <c r="F64" s="8">
         <v>46191</v>
       </c>
-      <c r="G64" s="18" t="s">
-        <v>14</v>
-      </c>
-      <c r="H64" s="20"/>
-      <c r="I64" s="16" t="s">
-        <v>125</v>
-      </c>
+      <c r="G64" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="H64" s="12"/>
+      <c r="I64" s="6"/>
       <c r="J64" s="6"/>
       <c r="K64" s="6"/>
       <c r="L64" s="21"/>
@@ -4158,12 +4158,12 @@
       <c r="Q64" s="21"/>
       <c r="R64" s="21"/>
       <c r="S64" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="65" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B65" s="6" t="s">
-        <v>10</v>
+        <v>99</v>
       </c>
       <c r="C65" s="6" t="s">
         <v>16</v>
@@ -4178,10 +4178,12 @@
       <c r="G65" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="H65" s="12"/>
+      <c r="H65" s="13"/>
       <c r="I65" s="6"/>
       <c r="J65" s="6"/>
-      <c r="K65" s="6"/>
+      <c r="K65" s="6" t="s">
+        <v>127</v>
+      </c>
       <c r="L65" s="21"/>
       <c r="M65" s="21"/>
       <c r="N65" s="21"/>
@@ -4190,31 +4192,33 @@
       <c r="Q65" s="21"/>
       <c r="R65" s="21"/>
       <c r="S65" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
     </row>
     <row r="66" spans="2:19" x14ac:dyDescent="0.35">
-      <c r="B66" s="6" t="s">
-        <v>99</v>
-      </c>
-      <c r="C66" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="D66" s="7"/>
-      <c r="E66" s="7" t="s">
+      <c r="B66" s="48" t="s">
+        <v>20</v>
+      </c>
+      <c r="C66" s="48" t="s">
+        <v>11</v>
+      </c>
+      <c r="D66" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="E66" s="9" t="s">
         <v>67</v>
       </c>
       <c r="F66" s="8">
         <v>46191</v>
       </c>
-      <c r="G66" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="H66" s="13"/>
+      <c r="G66" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="H66" s="12"/>
       <c r="I66" s="6"/>
       <c r="J66" s="6"/>
       <c r="K66" s="6" t="s">
-        <v>128</v>
+        <v>30</v>
       </c>
       <c r="L66" s="21"/>
       <c r="M66" s="21"/>
@@ -4224,33 +4228,33 @@
       <c r="Q66" s="21"/>
       <c r="R66" s="21"/>
       <c r="S66" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
     </row>
     <row r="67" spans="2:19" x14ac:dyDescent="0.35">
-      <c r="B67" s="48" t="s">
-        <v>20</v>
-      </c>
-      <c r="C67" s="48" t="s">
-        <v>11</v>
-      </c>
-      <c r="D67" s="9" t="s">
-        <v>12</v>
-      </c>
-      <c r="E67" s="9" t="s">
+      <c r="B67" s="6" t="s">
+        <v>99</v>
+      </c>
+      <c r="C67" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="D67" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="E67" s="7" t="s">
         <v>67</v>
       </c>
       <c r="F67" s="8">
-        <v>46191</v>
-      </c>
-      <c r="G67" s="9" t="s">
+        <v>46194</v>
+      </c>
+      <c r="G67" s="7" t="s">
         <v>14</v>
       </c>
       <c r="H67" s="12"/>
       <c r="I67" s="6"/>
       <c r="J67" s="6"/>
       <c r="K67" s="6" t="s">
-        <v>30</v>
+        <v>130</v>
       </c>
       <c r="L67" s="21"/>
       <c r="M67" s="21"/>
@@ -4260,24 +4264,24 @@
       <c r="Q67" s="21"/>
       <c r="R67" s="21"/>
       <c r="S67" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
     </row>
     <row r="68" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B68" s="6" t="s">
-        <v>99</v>
+        <v>10</v>
       </c>
       <c r="C68" s="6" t="s">
         <v>16</v>
       </c>
       <c r="D68" s="7" t="s">
-        <v>21</v>
+        <v>12</v>
       </c>
       <c r="E68" s="7" t="s">
         <v>67</v>
       </c>
       <c r="F68" s="8">
-        <v>46194</v>
+        <v>46195</v>
       </c>
       <c r="G68" s="7" t="s">
         <v>14</v>
@@ -4286,7 +4290,7 @@
       <c r="I68" s="6"/>
       <c r="J68" s="6"/>
       <c r="K68" s="6" t="s">
-        <v>131</v>
+        <v>50</v>
       </c>
       <c r="L68" s="21"/>
       <c r="M68" s="21"/>
@@ -4296,24 +4300,24 @@
       <c r="Q68" s="21"/>
       <c r="R68" s="21"/>
       <c r="S68" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
     </row>
     <row r="69" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B69" s="6" t="s">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="C69" s="6" t="s">
         <v>16</v>
       </c>
       <c r="D69" s="7" t="s">
-        <v>12</v>
+        <v>132</v>
       </c>
       <c r="E69" s="7" t="s">
         <v>67</v>
       </c>
-      <c r="F69" s="8">
-        <v>46195</v>
+      <c r="F69" s="11">
+        <v>46196</v>
       </c>
       <c r="G69" s="7" t="s">
         <v>14</v>
@@ -4321,9 +4325,7 @@
       <c r="H69" s="12"/>
       <c r="I69" s="6"/>
       <c r="J69" s="6"/>
-      <c r="K69" s="6" t="s">
-        <v>50</v>
-      </c>
+      <c r="K69" s="6"/>
       <c r="L69" s="21"/>
       <c r="M69" s="21"/>
       <c r="N69" s="21"/>
@@ -4332,32 +4334,38 @@
       <c r="Q69" s="21"/>
       <c r="R69" s="21"/>
       <c r="S69" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="70" spans="2:19" x14ac:dyDescent="0.35">
-      <c r="B70" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="C70" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="D70" s="7" t="s">
-        <v>134</v>
-      </c>
-      <c r="E70" s="7" t="s">
+      <c r="B70" s="21" t="s">
+        <v>99</v>
+      </c>
+      <c r="C70" s="21" t="s">
+        <v>11</v>
+      </c>
+      <c r="D70" s="44" t="s">
+        <v>217</v>
+      </c>
+      <c r="E70" s="24" t="s">
         <v>67</v>
       </c>
-      <c r="F70" s="11">
+      <c r="F70" s="25">
         <v>46196</v>
       </c>
-      <c r="G70" s="7" t="s">
+      <c r="G70" s="24" t="s">
         <v>14</v>
       </c>
       <c r="H70" s="12"/>
-      <c r="I70" s="6"/>
-      <c r="J70" s="6"/>
-      <c r="K70" s="6"/>
+      <c r="I70" s="21" t="s">
+        <v>70</v>
+      </c>
+      <c r="J70" s="44" t="s">
+        <v>218</v>
+      </c>
+      <c r="K70" s="44" t="s">
+        <v>214</v>
+      </c>
       <c r="L70" s="21"/>
       <c r="M70" s="21"/>
       <c r="N70" s="21"/>
@@ -4366,38 +4374,34 @@
       <c r="Q70" s="21"/>
       <c r="R70" s="21"/>
       <c r="S70" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
     <row r="71" spans="2:19" x14ac:dyDescent="0.35">
-      <c r="B71" s="21" t="s">
-        <v>99</v>
-      </c>
-      <c r="C71" s="21" t="s">
-        <v>11</v>
-      </c>
-      <c r="D71" s="44" t="s">
-        <v>219</v>
-      </c>
-      <c r="E71" s="24" t="s">
+      <c r="B71" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="C71" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="D71" s="7" t="s">
+        <v>73</v>
+      </c>
+      <c r="E71" s="7" t="s">
         <v>67</v>
       </c>
-      <c r="F71" s="25">
+      <c r="F71" s="8">
         <v>46196</v>
       </c>
-      <c r="G71" s="24" t="s">
+      <c r="G71" s="7" t="s">
         <v>14</v>
       </c>
       <c r="H71" s="12"/>
-      <c r="I71" s="21" t="s">
-        <v>70</v>
-      </c>
-      <c r="J71" s="44" t="s">
-        <v>220</v>
-      </c>
-      <c r="K71" s="44" t="s">
-        <v>216</v>
-      </c>
+      <c r="I71" s="6" t="s">
+        <v>135</v>
+      </c>
+      <c r="J71" s="6"/>
+      <c r="K71" s="6"/>
       <c r="L71" s="21"/>
       <c r="M71" s="21"/>
       <c r="N71" s="21"/>
@@ -4411,13 +4415,13 @@
     </row>
     <row r="72" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B72" s="6" t="s">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="C72" s="6" t="s">
         <v>16</v>
       </c>
       <c r="D72" s="7" t="s">
-        <v>73</v>
+        <v>21</v>
       </c>
       <c r="E72" s="7" t="s">
         <v>67</v>
@@ -4429,11 +4433,11 @@
         <v>14</v>
       </c>
       <c r="H72" s="12"/>
-      <c r="I72" s="6" t="s">
+      <c r="I72" s="50"/>
+      <c r="J72" s="6"/>
+      <c r="K72" s="6" t="s">
         <v>137</v>
       </c>
-      <c r="J72" s="6"/>
-      <c r="K72" s="6"/>
       <c r="L72" s="21"/>
       <c r="M72" s="21"/>
       <c r="N72" s="21"/>
@@ -4442,7 +4446,7 @@
       <c r="Q72" s="21"/>
       <c r="R72" s="21"/>
       <c r="S72" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="73" spans="2:19" x14ac:dyDescent="0.35">
@@ -4450,26 +4454,26 @@
         <v>20</v>
       </c>
       <c r="C73" s="6" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="D73" s="7" t="s">
-        <v>21</v>
+        <v>35</v>
       </c>
       <c r="E73" s="7" t="s">
         <v>67</v>
       </c>
       <c r="F73" s="8">
-        <v>46196</v>
+        <v>46198</v>
       </c>
       <c r="G73" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="H73" s="12"/>
-      <c r="I73" s="50"/>
+      <c r="H73" s="13"/>
+      <c r="I73" s="6" t="s">
+        <v>70</v>
+      </c>
       <c r="J73" s="6"/>
-      <c r="K73" s="6" t="s">
-        <v>139</v>
-      </c>
+      <c r="K73" s="6"/>
       <c r="L73" s="21"/>
       <c r="M73" s="21"/>
       <c r="N73" s="21"/>
@@ -4478,7 +4482,7 @@
       <c r="Q73" s="21"/>
       <c r="R73" s="21"/>
       <c r="S73" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="74" spans="2:19" x14ac:dyDescent="0.35">
@@ -4486,10 +4490,10 @@
         <v>20</v>
       </c>
       <c r="C74" s="6" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="D74" s="7" t="s">
-        <v>35</v>
+        <v>12</v>
       </c>
       <c r="E74" s="7" t="s">
         <v>67</v>
@@ -4498,12 +4502,12 @@
         <v>46198</v>
       </c>
       <c r="G74" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="H74" s="13"/>
-      <c r="I74" s="6" t="s">
-        <v>70</v>
-      </c>
+        <v>68</v>
+      </c>
+      <c r="H74" s="12">
+        <v>46253</v>
+      </c>
+      <c r="I74" s="6"/>
       <c r="J74" s="6"/>
       <c r="K74" s="6"/>
       <c r="L74" s="21"/>
@@ -4518,30 +4522,30 @@
       </c>
     </row>
     <row r="75" spans="2:19" x14ac:dyDescent="0.35">
-      <c r="B75" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="C75" s="6" t="s">
+      <c r="B75" s="47" t="s">
+        <v>10</v>
+      </c>
+      <c r="C75" s="47" t="s">
         <v>16</v>
       </c>
-      <c r="D75" s="7" t="s">
-        <v>12</v>
-      </c>
+      <c r="D75" s="7"/>
       <c r="E75" s="7" t="s">
         <v>67</v>
       </c>
-      <c r="F75" s="8">
+      <c r="F75" s="19">
         <v>46198</v>
       </c>
       <c r="G75" s="7" t="s">
-        <v>68</v>
-      </c>
-      <c r="H75" s="12">
-        <v>46253</v>
-      </c>
-      <c r="I75" s="6"/>
+        <v>14</v>
+      </c>
+      <c r="H75" s="22"/>
+      <c r="I75" s="6" t="s">
+        <v>61</v>
+      </c>
       <c r="J75" s="6"/>
-      <c r="K75" s="6"/>
+      <c r="K75" s="6" t="s">
+        <v>50</v>
+      </c>
       <c r="L75" s="21"/>
       <c r="M75" s="21"/>
       <c r="N75" s="21"/>
@@ -4550,34 +4554,32 @@
       <c r="Q75" s="21"/>
       <c r="R75" s="21"/>
       <c r="S75" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
     </row>
     <row r="76" spans="2:19" x14ac:dyDescent="0.35">
-      <c r="B76" s="47" t="s">
+      <c r="B76" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="C76" s="47" t="s">
-        <v>16</v>
-      </c>
-      <c r="D76" s="7"/>
+      <c r="C76" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="D76" s="7" t="s">
+        <v>21</v>
+      </c>
       <c r="E76" s="7" t="s">
         <v>67</v>
       </c>
-      <c r="F76" s="19">
+      <c r="F76" s="8">
         <v>46198</v>
       </c>
       <c r="G76" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="H76" s="22"/>
-      <c r="I76" s="6" t="s">
-        <v>61</v>
-      </c>
+      <c r="H76" s="12"/>
+      <c r="I76" s="6"/>
       <c r="J76" s="6"/>
-      <c r="K76" s="6" t="s">
-        <v>50</v>
-      </c>
+      <c r="K76" s="6"/>
       <c r="L76" s="21"/>
       <c r="M76" s="21"/>
       <c r="N76" s="21"/>
@@ -4586,7 +4588,7 @@
       <c r="Q76" s="21"/>
       <c r="R76" s="21"/>
       <c r="S76" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="77" spans="2:19" x14ac:dyDescent="0.35">
@@ -4597,21 +4599,27 @@
         <v>11</v>
       </c>
       <c r="D77" s="7" t="s">
-        <v>21</v>
+        <v>73</v>
       </c>
       <c r="E77" s="7" t="s">
         <v>67</v>
       </c>
       <c r="F77" s="8">
-        <v>46198</v>
+        <v>46202</v>
       </c>
       <c r="G77" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="H77" s="12"/>
-      <c r="I77" s="6"/>
+        <v>68</v>
+      </c>
+      <c r="H77" s="12">
+        <v>46252</v>
+      </c>
+      <c r="I77" s="6" t="s">
+        <v>143</v>
+      </c>
       <c r="J77" s="6"/>
-      <c r="K77" s="6"/>
+      <c r="K77" s="6" t="s">
+        <v>144</v>
+      </c>
       <c r="L77" s="21"/>
       <c r="M77" s="21"/>
       <c r="N77" s="21"/>
@@ -4620,15 +4628,15 @@
       <c r="Q77" s="21"/>
       <c r="R77" s="21"/>
       <c r="S77" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
     </row>
     <row r="78" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B78" s="6" t="s">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="C78" s="6" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="D78" s="7" t="s">
         <v>73</v>
@@ -4640,18 +4648,12 @@
         <v>46202</v>
       </c>
       <c r="G78" s="7" t="s">
-        <v>68</v>
-      </c>
-      <c r="H78" s="12">
-        <v>46252</v>
-      </c>
-      <c r="I78" s="6" t="s">
-        <v>145</v>
-      </c>
+        <v>14</v>
+      </c>
+      <c r="H78" s="12"/>
+      <c r="I78" s="6"/>
       <c r="J78" s="6"/>
-      <c r="K78" s="6" t="s">
-        <v>146</v>
-      </c>
+      <c r="K78" s="6"/>
       <c r="L78" s="21"/>
       <c r="M78" s="21"/>
       <c r="N78" s="21"/>
@@ -4660,7 +4662,7 @@
       <c r="Q78" s="21"/>
       <c r="R78" s="21"/>
       <c r="S78" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
     </row>
     <row r="79" spans="2:19" x14ac:dyDescent="0.35">
@@ -4671,19 +4673,21 @@
         <v>16</v>
       </c>
       <c r="D79" s="7" t="s">
-        <v>73</v>
+        <v>21</v>
       </c>
       <c r="E79" s="7" t="s">
         <v>67</v>
       </c>
-      <c r="F79" s="8">
-        <v>46202</v>
-      </c>
-      <c r="G79" s="7" t="s">
+      <c r="F79" s="11">
+        <v>46203</v>
+      </c>
+      <c r="G79" s="23" t="s">
         <v>14</v>
       </c>
       <c r="H79" s="12"/>
-      <c r="I79" s="6"/>
+      <c r="I79" s="6" t="s">
+        <v>39</v>
+      </c>
       <c r="J79" s="6"/>
       <c r="K79" s="6"/>
       <c r="L79" s="21"/>
@@ -4699,26 +4703,26 @@
     </row>
     <row r="80" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B80" s="6" t="s">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="C80" s="6" t="s">
         <v>16</v>
       </c>
       <c r="D80" s="7" t="s">
-        <v>21</v>
+        <v>12</v>
       </c>
       <c r="E80" s="7" t="s">
         <v>67</v>
       </c>
-      <c r="F80" s="11">
+      <c r="F80" s="8">
         <v>46203</v>
       </c>
-      <c r="G80" s="23" t="s">
-        <v>14</v>
-      </c>
-      <c r="H80" s="12"/>
+      <c r="G80" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="H80" s="13"/>
       <c r="I80" s="6" t="s">
-        <v>39</v>
+        <v>107</v>
       </c>
       <c r="J80" s="6"/>
       <c r="K80" s="6"/>
@@ -4730,7 +4734,7 @@
       <c r="Q80" s="21"/>
       <c r="R80" s="21"/>
       <c r="S80" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
     </row>
     <row r="81" spans="1:19" x14ac:dyDescent="0.35">
@@ -4740,9 +4744,7 @@
       <c r="C81" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="D81" s="7" t="s">
-        <v>12</v>
-      </c>
+      <c r="D81" s="7"/>
       <c r="E81" s="7" t="s">
         <v>67</v>
       </c>
@@ -4752,9 +4754,9 @@
       <c r="G81" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="H81" s="13"/>
+      <c r="H81" s="12"/>
       <c r="I81" s="6" t="s">
-        <v>107</v>
+        <v>70</v>
       </c>
       <c r="J81" s="6"/>
       <c r="K81" s="6"/>
@@ -4766,29 +4768,31 @@
       <c r="Q81" s="21"/>
       <c r="R81" s="21"/>
       <c r="S81" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="82" spans="1:19" x14ac:dyDescent="0.35">
       <c r="B82" s="6" t="s">
-        <v>10</v>
+        <v>63</v>
       </c>
       <c r="C82" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="D82" s="7"/>
+        <v>11</v>
+      </c>
+      <c r="D82" s="7" t="s">
+        <v>73</v>
+      </c>
       <c r="E82" s="7" t="s">
-        <v>67</v>
+        <v>150</v>
       </c>
       <c r="F82" s="8">
-        <v>46203</v>
+        <v>46204</v>
       </c>
       <c r="G82" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="H82" s="12"/>
+      <c r="H82" s="13"/>
       <c r="I82" s="6" t="s">
-        <v>70</v>
+        <v>29</v>
       </c>
       <c r="J82" s="6"/>
       <c r="K82" s="6"/>
@@ -4800,21 +4804,19 @@
       <c r="Q82" s="21"/>
       <c r="R82" s="21"/>
       <c r="S82" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="83" spans="1:19" x14ac:dyDescent="0.35">
       <c r="B83" s="6" t="s">
-        <v>63</v>
+        <v>10</v>
       </c>
       <c r="C83" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="D83" s="7" t="s">
-        <v>73</v>
-      </c>
+        <v>16</v>
+      </c>
+      <c r="D83" s="7"/>
       <c r="E83" s="7" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="F83" s="8">
         <v>46204</v>
@@ -4822,10 +4824,8 @@
       <c r="G83" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="H83" s="13"/>
-      <c r="I83" s="6" t="s">
-        <v>29</v>
-      </c>
+      <c r="H83" s="12"/>
+      <c r="I83" s="6"/>
       <c r="J83" s="6"/>
       <c r="K83" s="6"/>
       <c r="L83" s="21"/>
@@ -4840,26 +4840,33 @@
       </c>
     </row>
     <row r="84" spans="1:19" x14ac:dyDescent="0.35">
-      <c r="B84" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="C84" s="6" t="s">
+      <c r="A84" s="45" t="s">
+        <v>252</v>
+      </c>
+      <c r="B84" s="21" t="s">
+        <v>63</v>
+      </c>
+      <c r="C84" s="21" t="s">
         <v>16</v>
       </c>
-      <c r="D84" s="7"/>
-      <c r="E84" s="7" t="s">
-        <v>152</v>
-      </c>
-      <c r="F84" s="8">
+      <c r="D84" s="34" t="s">
+        <v>254</v>
+      </c>
+      <c r="E84" s="24" t="s">
+        <v>150</v>
+      </c>
+      <c r="F84" s="25">
         <v>46204</v>
       </c>
-      <c r="G84" s="7" t="s">
+      <c r="G84" s="24" t="s">
         <v>14</v>
       </c>
       <c r="H84" s="12"/>
-      <c r="I84" s="6"/>
-      <c r="J84" s="6"/>
-      <c r="K84" s="6"/>
+      <c r="I84" s="44"/>
+      <c r="J84" s="51" t="s">
+        <v>253</v>
+      </c>
+      <c r="K84" s="21"/>
       <c r="L84" s="21"/>
       <c r="M84" s="21"/>
       <c r="N84" s="21"/>
@@ -4872,32 +4879,27 @@
       </c>
     </row>
     <row r="85" spans="1:19" x14ac:dyDescent="0.35">
-      <c r="A85" s="45" t="s">
-        <v>254</v>
-      </c>
       <c r="B85" s="21" t="s">
-        <v>63</v>
+        <v>58</v>
       </c>
       <c r="C85" s="21" t="s">
-        <v>16</v>
-      </c>
-      <c r="D85" s="34" t="s">
-        <v>256</v>
-      </c>
+        <v>11</v>
+      </c>
+      <c r="D85" s="24"/>
       <c r="E85" s="24" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="F85" s="25">
-        <v>46204</v>
+        <v>46205</v>
       </c>
       <c r="G85" s="24" t="s">
         <v>14</v>
       </c>
       <c r="H85" s="12"/>
-      <c r="I85" s="44"/>
-      <c r="J85" s="51" t="s">
-        <v>255</v>
-      </c>
+      <c r="I85" s="21" t="s">
+        <v>74</v>
+      </c>
+      <c r="J85" s="21"/>
       <c r="K85" s="21"/>
       <c r="L85" s="21"/>
       <c r="M85" s="21"/>
@@ -4911,28 +4913,32 @@
       </c>
     </row>
     <row r="86" spans="1:19" x14ac:dyDescent="0.35">
-      <c r="B86" s="21" t="s">
-        <v>58</v>
-      </c>
-      <c r="C86" s="21" t="s">
-        <v>11</v>
-      </c>
-      <c r="D86" s="24"/>
-      <c r="E86" s="24" t="s">
-        <v>152</v>
-      </c>
-      <c r="F86" s="25">
-        <v>46205</v>
-      </c>
-      <c r="G86" s="24" t="s">
-        <v>14</v>
-      </c>
-      <c r="H86" s="12"/>
-      <c r="I86" s="21" t="s">
-        <v>74</v>
-      </c>
-      <c r="J86" s="21"/>
-      <c r="K86" s="21"/>
+      <c r="B86" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="C86" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="D86" s="26" t="s">
+        <v>12</v>
+      </c>
+      <c r="E86" s="26" t="s">
+        <v>150</v>
+      </c>
+      <c r="F86" s="27">
+        <v>46210</v>
+      </c>
+      <c r="G86" s="26" t="s">
+        <v>68</v>
+      </c>
+      <c r="H86" s="49"/>
+      <c r="I86" s="16" t="s">
+        <v>154</v>
+      </c>
+      <c r="J86" s="6"/>
+      <c r="K86" s="36" t="s">
+        <v>119</v>
+      </c>
       <c r="L86" s="21"/>
       <c r="M86" s="21"/>
       <c r="N86" s="21"/>
@@ -4945,32 +4951,28 @@
       </c>
     </row>
     <row r="87" spans="1:19" x14ac:dyDescent="0.35">
-      <c r="B87" s="16" t="s">
+      <c r="B87" s="21" t="s">
         <v>10</v>
       </c>
-      <c r="C87" s="16" t="s">
+      <c r="C87" s="21" t="s">
         <v>16</v>
       </c>
-      <c r="D87" s="26" t="s">
+      <c r="D87" s="24" t="s">
         <v>12</v>
       </c>
-      <c r="E87" s="26" t="s">
-        <v>152</v>
-      </c>
-      <c r="F87" s="27">
-        <v>46210</v>
-      </c>
-      <c r="G87" s="26" t="s">
-        <v>68</v>
-      </c>
-      <c r="H87" s="49"/>
-      <c r="I87" s="16" t="s">
-        <v>156</v>
-      </c>
-      <c r="J87" s="6"/>
-      <c r="K87" s="36" t="s">
-        <v>120</v>
-      </c>
+      <c r="E87" s="24" t="s">
+        <v>150</v>
+      </c>
+      <c r="F87" s="25">
+        <v>46211</v>
+      </c>
+      <c r="G87" s="24" t="s">
+        <v>14</v>
+      </c>
+      <c r="H87" s="12"/>
+      <c r="I87" s="21"/>
+      <c r="J87" s="21"/>
+      <c r="K87" s="21"/>
       <c r="L87" s="21"/>
       <c r="M87" s="21"/>
       <c r="N87" s="21"/>
@@ -4979,24 +4981,24 @@
       <c r="Q87" s="21"/>
       <c r="R87" s="21"/>
       <c r="S87" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
     </row>
     <row r="88" spans="1:19" x14ac:dyDescent="0.35">
       <c r="B88" s="21" t="s">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="C88" s="21" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="D88" s="24" t="s">
-        <v>12</v>
+        <v>21</v>
       </c>
       <c r="E88" s="24" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="F88" s="25">
-        <v>46211</v>
+        <v>46212</v>
       </c>
       <c r="G88" s="24" t="s">
         <v>14</v>
@@ -5018,16 +5020,16 @@
     </row>
     <row r="89" spans="1:19" x14ac:dyDescent="0.35">
       <c r="B89" s="21" t="s">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="C89" s="21" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="D89" s="24" t="s">
-        <v>21</v>
+        <v>12</v>
       </c>
       <c r="E89" s="24" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="F89" s="25">
         <v>46212</v>
@@ -5052,26 +5054,32 @@
     </row>
     <row r="90" spans="1:19" x14ac:dyDescent="0.35">
       <c r="B90" s="21" t="s">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="C90" s="21" t="s">
         <v>16</v>
       </c>
       <c r="D90" s="24" t="s">
-        <v>12</v>
+        <v>132</v>
       </c>
       <c r="E90" s="24" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="F90" s="25">
         <v>46212</v>
       </c>
       <c r="G90" s="24" t="s">
-        <v>14</v>
-      </c>
-      <c r="H90" s="12"/>
-      <c r="I90" s="21"/>
-      <c r="J90" s="21"/>
+        <v>68</v>
+      </c>
+      <c r="H90" s="22">
+        <v>46259</v>
+      </c>
+      <c r="I90" s="21" t="s">
+        <v>159</v>
+      </c>
+      <c r="J90" s="21" t="s">
+        <v>160</v>
+      </c>
       <c r="K90" s="21"/>
       <c r="L90" s="21"/>
       <c r="M90" s="21"/>
@@ -5086,16 +5094,16 @@
     </row>
     <row r="91" spans="1:19" x14ac:dyDescent="0.35">
       <c r="B91" s="21" t="s">
-        <v>20</v>
+        <v>58</v>
       </c>
       <c r="C91" s="21" t="s">
         <v>16</v>
       </c>
-      <c r="D91" s="24" t="s">
-        <v>134</v>
+      <c r="D91" s="44" t="s">
+        <v>251</v>
       </c>
       <c r="E91" s="24" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="F91" s="25">
         <v>46212</v>
@@ -5104,15 +5112,17 @@
         <v>68</v>
       </c>
       <c r="H91" s="22">
-        <v>46259</v>
+        <v>46258</v>
       </c>
       <c r="I91" s="21" t="s">
-        <v>161</v>
-      </c>
-      <c r="J91" s="21" t="s">
         <v>162</v>
       </c>
-      <c r="K91" s="21"/>
+      <c r="J91" s="44" t="s">
+        <v>251</v>
+      </c>
+      <c r="K91" s="44" t="s">
+        <v>250</v>
+      </c>
       <c r="L91" s="21"/>
       <c r="M91" s="21"/>
       <c r="N91" s="21"/>
@@ -5121,39 +5131,37 @@
       <c r="Q91" s="21"/>
       <c r="R91" s="21"/>
       <c r="S91" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
     </row>
     <row r="92" spans="1:19" x14ac:dyDescent="0.35">
       <c r="B92" s="21" t="s">
-        <v>58</v>
+        <v>10</v>
       </c>
       <c r="C92" s="21" t="s">
-        <v>16</v>
-      </c>
-      <c r="D92" s="44" t="s">
-        <v>253</v>
+        <v>11</v>
+      </c>
+      <c r="D92" s="24" t="s">
+        <v>12</v>
       </c>
       <c r="E92" s="24" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="F92" s="25">
         <v>46212</v>
       </c>
       <c r="G92" s="24" t="s">
-        <v>68</v>
-      </c>
-      <c r="H92" s="22">
-        <v>46258</v>
+        <v>89</v>
+      </c>
+      <c r="H92" s="12">
+        <v>46259</v>
       </c>
       <c r="I92" s="21" t="s">
         <v>164</v>
       </c>
-      <c r="J92" s="44" t="s">
-        <v>253</v>
-      </c>
-      <c r="K92" s="44" t="s">
-        <v>252</v>
+      <c r="J92" s="21"/>
+      <c r="K92" s="53" t="s">
+        <v>165</v>
       </c>
       <c r="L92" s="21"/>
       <c r="M92" s="21"/>
@@ -5163,38 +5171,33 @@
       <c r="Q92" s="21"/>
       <c r="R92" s="21"/>
       <c r="S92" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
     </row>
     <row r="93" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="A93" s="45" t="s">
+        <v>255</v>
+      </c>
       <c r="B93" s="21" t="s">
         <v>10</v>
       </c>
       <c r="C93" s="21" t="s">
-        <v>11</v>
-      </c>
-      <c r="D93" s="24" t="s">
-        <v>12</v>
-      </c>
+        <v>207</v>
+      </c>
+      <c r="D93" s="44"/>
       <c r="E93" s="24" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="F93" s="25">
         <v>46212</v>
       </c>
       <c r="G93" s="24" t="s">
-        <v>89</v>
-      </c>
-      <c r="H93" s="12">
-        <v>46259</v>
-      </c>
-      <c r="I93" s="21" t="s">
-        <v>166</v>
-      </c>
-      <c r="J93" s="21"/>
-      <c r="K93" s="53" t="s">
-        <v>167</v>
-      </c>
+        <v>14</v>
+      </c>
+      <c r="H93" s="12"/>
+      <c r="I93" s="44"/>
+      <c r="J93" s="44"/>
+      <c r="K93" s="21"/>
       <c r="L93" s="21"/>
       <c r="M93" s="21"/>
       <c r="N93" s="21"/>
@@ -5207,28 +5210,25 @@
       </c>
     </row>
     <row r="94" spans="1:19" x14ac:dyDescent="0.35">
-      <c r="A94" s="45" t="s">
-        <v>257</v>
-      </c>
       <c r="B94" s="21" t="s">
         <v>10</v>
       </c>
       <c r="C94" s="21" t="s">
-        <v>209</v>
-      </c>
-      <c r="D94" s="44"/>
+        <v>11</v>
+      </c>
+      <c r="D94" s="24"/>
       <c r="E94" s="24" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="F94" s="25">
-        <v>46212</v>
+        <v>46216</v>
       </c>
       <c r="G94" s="24" t="s">
         <v>14</v>
       </c>
       <c r="H94" s="12"/>
-      <c r="I94" s="44"/>
-      <c r="J94" s="44"/>
+      <c r="I94" s="21"/>
+      <c r="J94" s="21"/>
       <c r="K94" s="21"/>
       <c r="L94" s="21"/>
       <c r="M94" s="21"/>
@@ -5243,14 +5243,16 @@
     </row>
     <row r="95" spans="1:19" x14ac:dyDescent="0.35">
       <c r="B95" s="21" t="s">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="C95" s="21" t="s">
         <v>11</v>
       </c>
-      <c r="D95" s="24"/>
+      <c r="D95" s="24" t="s">
+        <v>73</v>
+      </c>
       <c r="E95" s="24" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="F95" s="25">
         <v>46216</v>
@@ -5258,8 +5260,10 @@
       <c r="G95" s="24" t="s">
         <v>14</v>
       </c>
-      <c r="H95" s="12"/>
-      <c r="I95" s="21"/>
+      <c r="H95" s="13"/>
+      <c r="I95" s="21" t="s">
+        <v>135</v>
+      </c>
       <c r="J95" s="21"/>
       <c r="K95" s="21"/>
       <c r="L95" s="21"/>
@@ -5270,33 +5274,35 @@
       <c r="Q95" s="21"/>
       <c r="R95" s="21"/>
       <c r="S95" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
     </row>
     <row r="96" spans="1:19" x14ac:dyDescent="0.35">
       <c r="B96" s="21" t="s">
-        <v>20</v>
+        <v>58</v>
       </c>
       <c r="C96" s="21" t="s">
         <v>11</v>
       </c>
       <c r="D96" s="24" t="s">
-        <v>73</v>
+        <v>12</v>
       </c>
       <c r="E96" s="24" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="F96" s="25">
-        <v>46216</v>
+        <v>46219</v>
       </c>
       <c r="G96" s="24" t="s">
         <v>14</v>
       </c>
-      <c r="H96" s="13"/>
+      <c r="H96" s="12"/>
       <c r="I96" s="21" t="s">
-        <v>137</v>
-      </c>
-      <c r="J96" s="21"/>
+        <v>169</v>
+      </c>
+      <c r="J96" s="44" t="s">
+        <v>220</v>
+      </c>
       <c r="K96" s="21"/>
       <c r="L96" s="21"/>
       <c r="M96" s="21"/>
@@ -5311,31 +5317,35 @@
     </row>
     <row r="97" spans="1:19" x14ac:dyDescent="0.35">
       <c r="B97" s="21" t="s">
-        <v>58</v>
+        <v>10</v>
       </c>
       <c r="C97" s="21" t="s">
         <v>11</v>
       </c>
-      <c r="D97" s="24" t="s">
-        <v>12</v>
+      <c r="D97" s="44" t="s">
+        <v>220</v>
       </c>
       <c r="E97" s="24" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="F97" s="25">
         <v>46219</v>
       </c>
       <c r="G97" s="24" t="s">
-        <v>14</v>
-      </c>
-      <c r="H97" s="12"/>
+        <v>89</v>
+      </c>
+      <c r="H97" s="22">
+        <v>46265</v>
+      </c>
       <c r="I97" s="21" t="s">
+        <v>164</v>
+      </c>
+      <c r="J97" s="44" t="s">
+        <v>219</v>
+      </c>
+      <c r="K97" s="21" t="s">
         <v>171</v>
       </c>
-      <c r="J97" s="44" t="s">
-        <v>222</v>
-      </c>
-      <c r="K97" s="21"/>
       <c r="L97" s="21"/>
       <c r="M97" s="21"/>
       <c r="N97" s="21"/>
@@ -5344,40 +5354,36 @@
       <c r="Q97" s="21"/>
       <c r="R97" s="21"/>
       <c r="S97" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
     </row>
     <row r="98" spans="1:19" x14ac:dyDescent="0.35">
       <c r="B98" s="21" t="s">
-        <v>10</v>
+        <v>58</v>
       </c>
       <c r="C98" s="21" t="s">
         <v>11</v>
       </c>
-      <c r="D98" s="44" t="s">
-        <v>222</v>
+      <c r="D98" s="24" t="s">
+        <v>173</v>
       </c>
       <c r="E98" s="24" t="s">
-        <v>152</v>
-      </c>
-      <c r="F98" s="25">
-        <v>46219</v>
+        <v>150</v>
+      </c>
+      <c r="F98" s="28">
+        <v>46223</v>
       </c>
       <c r="G98" s="24" t="s">
-        <v>89</v>
-      </c>
-      <c r="H98" s="22">
-        <v>46265</v>
-      </c>
+        <v>14</v>
+      </c>
+      <c r="H98" s="12"/>
       <c r="I98" s="21" t="s">
-        <v>166</v>
-      </c>
-      <c r="J98" s="44" t="s">
-        <v>221</v>
-      </c>
-      <c r="K98" s="21" t="s">
+        <v>29</v>
+      </c>
+      <c r="J98" s="21" t="s">
         <v>173</v>
       </c>
+      <c r="K98" s="21"/>
       <c r="L98" s="21"/>
       <c r="M98" s="21"/>
       <c r="N98" s="21"/>
@@ -5386,23 +5392,23 @@
       <c r="Q98" s="21"/>
       <c r="R98" s="21"/>
       <c r="S98" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
     </row>
     <row r="99" spans="1:19" x14ac:dyDescent="0.35">
       <c r="B99" s="21" t="s">
-        <v>58</v>
+        <v>20</v>
       </c>
       <c r="C99" s="21" t="s">
         <v>11</v>
       </c>
       <c r="D99" s="24" t="s">
-        <v>175</v>
+        <v>21</v>
       </c>
       <c r="E99" s="24" t="s">
-        <v>152</v>
-      </c>
-      <c r="F99" s="28">
+        <v>150</v>
+      </c>
+      <c r="F99" s="25">
         <v>46223</v>
       </c>
       <c r="G99" s="24" t="s">
@@ -5410,11 +5416,9 @@
       </c>
       <c r="H99" s="12"/>
       <c r="I99" s="21" t="s">
-        <v>29</v>
-      </c>
-      <c r="J99" s="21" t="s">
         <v>175</v>
       </c>
+      <c r="J99" s="21"/>
       <c r="K99" s="21"/>
       <c r="L99" s="21"/>
       <c r="M99" s="21"/>
@@ -5424,34 +5428,36 @@
       <c r="Q99" s="21"/>
       <c r="R99" s="21"/>
       <c r="S99" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
     </row>
     <row r="100" spans="1:19" x14ac:dyDescent="0.35">
-      <c r="B100" s="21" t="s">
-        <v>20</v>
-      </c>
-      <c r="C100" s="21" t="s">
+      <c r="B100" s="6" t="s">
+        <v>99</v>
+      </c>
+      <c r="C100" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="D100" s="24" t="s">
-        <v>21</v>
-      </c>
-      <c r="E100" s="24" t="s">
-        <v>152</v>
-      </c>
-      <c r="F100" s="25">
-        <v>46223</v>
-      </c>
-      <c r="G100" s="24" t="s">
+      <c r="D100" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="E100" s="7" t="s">
+        <v>150</v>
+      </c>
+      <c r="F100" s="8">
+        <v>46224</v>
+      </c>
+      <c r="G100" s="7" t="s">
         <v>14</v>
       </c>
       <c r="H100" s="12"/>
-      <c r="I100" s="21" t="s">
+      <c r="I100" s="6"/>
+      <c r="J100" s="6" t="s">
         <v>177</v>
       </c>
-      <c r="J100" s="21"/>
-      <c r="K100" s="21"/>
+      <c r="K100" s="6" t="s">
+        <v>178</v>
+      </c>
       <c r="L100" s="21"/>
       <c r="M100" s="21"/>
       <c r="N100" s="21"/>
@@ -5460,35 +5466,40 @@
       <c r="Q100" s="21"/>
       <c r="R100" s="21"/>
       <c r="S100" t="s">
-        <v>211</v>
+        <v>262</v>
       </c>
     </row>
     <row r="101" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="A101" s="41" t="s">
+        <v>256</v>
+      </c>
       <c r="B101" s="6" t="s">
-        <v>99</v>
+        <v>20</v>
       </c>
       <c r="C101" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="D101" s="7" t="s">
-        <v>32</v>
+        <v>16</v>
+      </c>
+      <c r="D101" s="34" t="s">
+        <v>257</v>
       </c>
       <c r="E101" s="7" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="F101" s="8">
         <v>46224</v>
       </c>
-      <c r="G101" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="H101" s="12"/>
-      <c r="I101" s="6"/>
-      <c r="J101" s="6" t="s">
-        <v>179</v>
-      </c>
-      <c r="K101" s="6" t="s">
-        <v>180</v>
+      <c r="G101" s="42" t="s">
+        <v>89</v>
+      </c>
+      <c r="H101" s="12">
+        <v>46274</v>
+      </c>
+      <c r="I101" s="34"/>
+      <c r="J101" s="34" t="s">
+        <v>257</v>
+      </c>
+      <c r="K101" s="34" t="s">
+        <v>258</v>
       </c>
       <c r="L101" s="21"/>
       <c r="M101" s="21"/>
@@ -5498,104 +5509,97 @@
       <c r="Q101" s="21"/>
       <c r="R101" s="21"/>
       <c r="S101" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
     </row>
     <row r="102" spans="1:19" x14ac:dyDescent="0.35">
-      <c r="A102" s="41" t="s">
-        <v>258</v>
-      </c>
       <c r="B102" s="6" t="s">
         <v>20</v>
       </c>
       <c r="C102" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="D102" s="34" t="s">
-        <v>259</v>
+        <v>11</v>
+      </c>
+      <c r="D102" s="7" t="s">
+        <v>180</v>
       </c>
       <c r="E102" s="7" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="F102" s="8">
-        <v>46224</v>
-      </c>
-      <c r="G102" s="42" t="s">
-        <v>89</v>
+        <v>46227</v>
+      </c>
+      <c r="G102" s="7" t="s">
+        <v>68</v>
       </c>
       <c r="H102" s="12">
-        <v>46274</v>
-      </c>
-      <c r="I102" s="34"/>
-      <c r="J102" s="34" t="s">
-        <v>259</v>
-      </c>
-      <c r="K102" s="34" t="s">
-        <v>260</v>
-      </c>
-      <c r="L102" s="21"/>
-      <c r="M102" s="21"/>
-      <c r="N102" s="21"/>
-      <c r="O102" s="21"/>
-      <c r="P102" s="21"/>
-      <c r="Q102" s="21"/>
-      <c r="R102" s="21"/>
+        <v>46255</v>
+      </c>
+      <c r="I102" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="J102" s="6" t="s">
+        <v>180</v>
+      </c>
+      <c r="K102" s="6"/>
+      <c r="L102" s="6"/>
+      <c r="M102" s="6"/>
+      <c r="N102" s="6"/>
+      <c r="O102" s="6"/>
+      <c r="P102" s="6"/>
+      <c r="Q102" s="6"/>
+      <c r="R102" s="6"/>
       <c r="S102" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
     </row>
     <row r="103" spans="1:19" x14ac:dyDescent="0.35">
       <c r="B103" s="6" t="s">
-        <v>20</v>
+        <v>99</v>
       </c>
       <c r="C103" s="6" t="s">
         <v>11</v>
       </c>
       <c r="D103" s="7" t="s">
-        <v>182</v>
+        <v>21</v>
       </c>
       <c r="E103" s="7" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="F103" s="8">
         <v>46227</v>
       </c>
       <c r="G103" s="7" t="s">
-        <v>68</v>
-      </c>
-      <c r="H103" s="12">
-        <v>46255</v>
-      </c>
+        <v>14</v>
+      </c>
+      <c r="H103" s="12"/>
       <c r="I103" s="6" t="s">
-        <v>104</v>
-      </c>
-      <c r="J103" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="J103" s="6"/>
+      <c r="K103" s="6" t="s">
         <v>182</v>
       </c>
-      <c r="K103" s="6"/>
-      <c r="L103" s="6"/>
-      <c r="M103" s="6"/>
-      <c r="N103" s="6"/>
-      <c r="O103" s="6"/>
-      <c r="P103" s="6"/>
-      <c r="Q103" s="6"/>
-      <c r="R103" s="6"/>
+      <c r="L103" s="21"/>
+      <c r="M103" s="21"/>
+      <c r="N103" s="21"/>
+      <c r="O103" s="21"/>
+      <c r="P103" s="21"/>
+      <c r="Q103" s="21"/>
+      <c r="R103" s="21"/>
       <c r="S103" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
     </row>
     <row r="104" spans="1:19" x14ac:dyDescent="0.35">
       <c r="B104" s="6" t="s">
-        <v>99</v>
+        <v>58</v>
       </c>
       <c r="C104" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="D104" s="7" t="s">
-        <v>21</v>
-      </c>
+        <v>16</v>
+      </c>
+      <c r="D104" s="7"/>
       <c r="E104" s="7" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="F104" s="8">
         <v>46227</v>
@@ -5604,9 +5608,7 @@
         <v>14</v>
       </c>
       <c r="H104" s="12"/>
-      <c r="I104" s="6" t="s">
-        <v>49</v>
-      </c>
+      <c r="I104" s="6"/>
       <c r="J104" s="6"/>
       <c r="K104" s="6" t="s">
         <v>184</v>
@@ -5619,19 +5621,21 @@
       <c r="Q104" s="21"/>
       <c r="R104" s="21"/>
       <c r="S104" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
     </row>
     <row r="105" spans="1:19" x14ac:dyDescent="0.35">
       <c r="B105" s="6" t="s">
-        <v>58</v>
+        <v>20</v>
       </c>
       <c r="C105" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="D105" s="7"/>
+      <c r="D105" s="7" t="s">
+        <v>12</v>
+      </c>
       <c r="E105" s="7" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="F105" s="8">
         <v>46227</v>
@@ -5640,10 +5644,12 @@
         <v>14</v>
       </c>
       <c r="H105" s="12"/>
-      <c r="I105" s="6"/>
+      <c r="I105" s="6" t="s">
+        <v>186</v>
+      </c>
       <c r="J105" s="6"/>
       <c r="K105" s="6" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="L105" s="21"/>
       <c r="M105" s="21"/>
@@ -5653,35 +5659,37 @@
       <c r="Q105" s="21"/>
       <c r="R105" s="21"/>
       <c r="S105" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
     </row>
     <row r="106" spans="1:19" x14ac:dyDescent="0.35">
       <c r="B106" s="6" t="s">
-        <v>20</v>
+        <v>99</v>
       </c>
       <c r="C106" s="6" t="s">
         <v>16</v>
       </c>
       <c r="D106" s="7" t="s">
-        <v>12</v>
+        <v>189</v>
       </c>
       <c r="E106" s="7" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="F106" s="8">
-        <v>46227</v>
+        <v>46231</v>
       </c>
       <c r="G106" s="7" t="s">
         <v>14</v>
       </c>
       <c r="H106" s="12"/>
       <c r="I106" s="6" t="s">
-        <v>188</v>
-      </c>
-      <c r="J106" s="6"/>
+        <v>190</v>
+      </c>
+      <c r="J106" s="6" t="s">
+        <v>189</v>
+      </c>
       <c r="K106" s="6" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="L106" s="21"/>
       <c r="M106" s="21"/>
@@ -5691,37 +5699,36 @@
       <c r="Q106" s="21"/>
       <c r="R106" s="21"/>
       <c r="S106" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
     </row>
     <row r="107" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="A107" s="46" t="s">
+        <v>260</v>
+      </c>
       <c r="B107" s="6" t="s">
-        <v>99</v>
+        <v>20</v>
       </c>
       <c r="C107" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="D107" s="7" t="s">
-        <v>191</v>
+        <v>11</v>
+      </c>
+      <c r="D107" s="34" t="s">
+        <v>259</v>
       </c>
       <c r="E107" s="7" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="F107" s="8">
-        <v>46231</v>
-      </c>
-      <c r="G107" s="7" t="s">
+        <v>46232</v>
+      </c>
+      <c r="G107" s="42" t="s">
         <v>14</v>
       </c>
       <c r="H107" s="12"/>
-      <c r="I107" s="6" t="s">
-        <v>192</v>
-      </c>
-      <c r="J107" s="6" t="s">
-        <v>191</v>
-      </c>
-      <c r="K107" s="6" t="s">
-        <v>193</v>
+      <c r="I107" s="34"/>
+      <c r="J107" s="34"/>
+      <c r="K107" s="35" t="s">
+        <v>261</v>
       </c>
       <c r="L107" s="21"/>
       <c r="M107" s="21"/>
@@ -5731,37 +5738,36 @@
       <c r="Q107" s="21"/>
       <c r="R107" s="21"/>
       <c r="S107" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="108" spans="1:19" x14ac:dyDescent="0.35">
-      <c r="A108" s="46" t="s">
-        <v>262</v>
-      </c>
       <c r="B108" s="6" t="s">
-        <v>20</v>
+        <v>99</v>
       </c>
       <c r="C108" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="D108" s="34" t="s">
-        <v>261</v>
+      <c r="D108" s="7" t="s">
+        <v>193</v>
       </c>
       <c r="E108" s="7" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="F108" s="8">
-        <v>46232</v>
-      </c>
-      <c r="G108" s="42" t="s">
+        <v>46233</v>
+      </c>
+      <c r="G108" s="7" t="s">
         <v>14</v>
       </c>
       <c r="H108" s="12"/>
-      <c r="I108" s="34"/>
-      <c r="J108" s="34"/>
-      <c r="K108" s="35" t="s">
-        <v>263</v>
-      </c>
+      <c r="I108" s="6" t="s">
+        <v>124</v>
+      </c>
+      <c r="J108" s="6" t="s">
+        <v>193</v>
+      </c>
+      <c r="K108" s="6"/>
       <c r="L108" s="21"/>
       <c r="M108" s="21"/>
       <c r="N108" s="21"/>
@@ -5770,32 +5776,30 @@
       <c r="Q108" s="21"/>
       <c r="R108" s="21"/>
       <c r="S108" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
     </row>
     <row r="109" spans="1:19" x14ac:dyDescent="0.35">
       <c r="B109" s="6" t="s">
-        <v>99</v>
+        <v>20</v>
       </c>
       <c r="C109" s="6" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="D109" s="7" t="s">
         <v>195</v>
       </c>
       <c r="E109" s="7" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="F109" s="8">
         <v>46233</v>
       </c>
       <c r="G109" s="7" t="s">
-        <v>14</v>
+        <v>68</v>
       </c>
       <c r="H109" s="12"/>
-      <c r="I109" s="6" t="s">
-        <v>125</v>
-      </c>
+      <c r="I109" s="6"/>
       <c r="J109" s="6" t="s">
         <v>195</v>
       </c>
@@ -5808,12 +5812,12 @@
       <c r="Q109" s="21"/>
       <c r="R109" s="21"/>
       <c r="S109" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
     </row>
     <row r="110" spans="1:19" x14ac:dyDescent="0.35">
       <c r="B110" s="6" t="s">
-        <v>20</v>
+        <v>99</v>
       </c>
       <c r="C110" s="6" t="s">
         <v>16</v>
@@ -5822,20 +5826,22 @@
         <v>197</v>
       </c>
       <c r="E110" s="7" t="s">
-        <v>152</v>
+        <v>198</v>
       </c>
       <c r="F110" s="8">
-        <v>46233</v>
+        <v>46244</v>
       </c>
       <c r="G110" s="7" t="s">
-        <v>68</v>
+        <v>14</v>
       </c>
       <c r="H110" s="12"/>
       <c r="I110" s="6"/>
       <c r="J110" s="6" t="s">
-        <v>197</v>
-      </c>
-      <c r="K110" s="6"/>
+        <v>199</v>
+      </c>
+      <c r="K110" s="6" t="s">
+        <v>30</v>
+      </c>
       <c r="L110" s="21"/>
       <c r="M110" s="21"/>
       <c r="N110" s="21"/>
@@ -5844,7 +5850,7 @@
       <c r="Q110" s="21"/>
       <c r="R110" s="21"/>
       <c r="S110" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
     </row>
     <row r="111" spans="1:19" x14ac:dyDescent="0.35">
@@ -5852,28 +5858,24 @@
         <v>99</v>
       </c>
       <c r="C111" s="6" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="D111" s="7" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="E111" s="7" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="F111" s="8">
-        <v>46244</v>
+        <v>46247</v>
       </c>
       <c r="G111" s="7" t="s">
         <v>14</v>
       </c>
       <c r="H111" s="12"/>
       <c r="I111" s="6"/>
-      <c r="J111" s="6" t="s">
-        <v>201</v>
-      </c>
-      <c r="K111" s="6" t="s">
-        <v>30</v>
-      </c>
+      <c r="J111" s="6"/>
+      <c r="K111" s="6"/>
       <c r="L111" s="21"/>
       <c r="M111" s="21"/>
       <c r="N111" s="21"/>
@@ -5882,21 +5884,19 @@
       <c r="Q111" s="21"/>
       <c r="R111" s="21"/>
       <c r="S111" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="112" spans="1:19" x14ac:dyDescent="0.35">
       <c r="B112" s="6" t="s">
-        <v>99</v>
+        <v>20</v>
       </c>
       <c r="C112" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="D112" s="7" t="s">
-        <v>203</v>
-      </c>
+        <v>16</v>
+      </c>
+      <c r="D112" s="7"/>
       <c r="E112" s="7" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="F112" s="8">
         <v>46247</v>
@@ -5916,29 +5916,35 @@
       <c r="Q112" s="21"/>
       <c r="R112" s="21"/>
       <c r="S112" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
     </row>
     <row r="113" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B113" s="6" t="s">
-        <v>20</v>
+        <v>99</v>
       </c>
       <c r="C113" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="D113" s="7"/>
+        <v>11</v>
+      </c>
+      <c r="D113" s="7" t="s">
+        <v>204</v>
+      </c>
       <c r="E113" s="7" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="F113" s="8">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="G113" s="7" t="s">
         <v>14</v>
       </c>
       <c r="H113" s="12"/>
-      <c r="I113" s="6"/>
-      <c r="J113" s="6"/>
+      <c r="I113" s="6" t="s">
+        <v>205</v>
+      </c>
+      <c r="J113" s="6" t="s">
+        <v>204</v>
+      </c>
       <c r="K113" s="6"/>
       <c r="L113" s="21"/>
       <c r="M113" s="21"/>
@@ -5948,34 +5954,34 @@
       <c r="Q113" s="21"/>
       <c r="R113" s="21"/>
       <c r="S113" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
     </row>
     <row r="114" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B114" s="6" t="s">
-        <v>99</v>
+        <v>10</v>
       </c>
       <c r="C114" s="6" t="s">
-        <v>11</v>
+        <v>207</v>
       </c>
       <c r="D114" s="7" t="s">
-        <v>206</v>
+        <v>12</v>
       </c>
       <c r="E114" s="7" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="F114" s="8">
-        <v>46248</v>
+        <v>46251</v>
       </c>
       <c r="G114" s="7" t="s">
         <v>14</v>
       </c>
       <c r="H114" s="12"/>
       <c r="I114" s="6" t="s">
-        <v>207</v>
-      </c>
-      <c r="J114" s="6" t="s">
-        <v>206</v>
+        <v>18</v>
+      </c>
+      <c r="J114" s="52" t="s">
+        <v>208</v>
       </c>
       <c r="K114" s="6"/>
       <c r="L114" s="21"/>
@@ -5986,46 +5992,27 @@
       <c r="Q114" s="21"/>
       <c r="R114" s="21"/>
       <c r="S114" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="115" spans="2:19" x14ac:dyDescent="0.35">
-      <c r="B115" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="C115" s="6" t="s">
-        <v>209</v>
-      </c>
-      <c r="D115" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="E115" s="7" t="s">
-        <v>200</v>
-      </c>
-      <c r="F115" s="8">
-        <v>46251</v>
-      </c>
-      <c r="G115" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="H115" s="12"/>
-      <c r="I115" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="J115" s="52" t="s">
-        <v>210</v>
-      </c>
-      <c r="K115" s="6"/>
-      <c r="L115" s="21"/>
-      <c r="M115" s="21"/>
-      <c r="N115" s="21"/>
-      <c r="O115" s="21"/>
-      <c r="P115" s="21"/>
-      <c r="Q115" s="21"/>
-      <c r="R115" s="21"/>
-      <c r="S115" t="s">
-        <v>278</v>
-      </c>
+      <c r="B115" s="29"/>
+      <c r="C115" s="29"/>
+      <c r="D115" s="30"/>
+      <c r="E115" s="30"/>
+      <c r="F115" s="31"/>
+      <c r="G115" s="30"/>
+      <c r="H115" s="32"/>
+      <c r="I115" s="29"/>
+      <c r="J115" s="29"/>
+      <c r="K115" s="29"/>
+      <c r="L115" s="29"/>
+      <c r="M115" s="29"/>
+      <c r="N115" s="29"/>
+      <c r="O115" s="29"/>
+      <c r="P115" s="29"/>
+      <c r="Q115" s="29"/>
+      <c r="R115" s="29"/>
     </row>
     <row r="116" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B116" s="29"/>
@@ -7509,56 +7496,37 @@
       <c r="Q193" s="29"/>
       <c r="R193" s="29"/>
     </row>
-    <row r="194" spans="2:18" x14ac:dyDescent="0.35">
-      <c r="B194" s="29"/>
-      <c r="C194" s="29"/>
-      <c r="D194" s="30"/>
-      <c r="E194" s="30"/>
-      <c r="F194" s="31"/>
-      <c r="G194" s="30"/>
-      <c r="H194" s="32"/>
-      <c r="I194" s="29"/>
-      <c r="J194" s="29"/>
-      <c r="K194" s="29"/>
-      <c r="L194" s="29"/>
-      <c r="M194" s="29"/>
-      <c r="N194" s="29"/>
-      <c r="O194" s="29"/>
-      <c r="P194" s="29"/>
-      <c r="Q194" s="29"/>
-      <c r="R194" s="29"/>
-    </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:L199">
-    <sortCondition ref="F2:F199"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:L198">
+    <sortCondition ref="F2:F198"/>
   </sortState>
   <phoneticPr fontId="13" type="noConversion"/>
   <dataValidations count="10">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D86:D100 D116:D1048576 D50:D59 D4:D28 D81:D84 D103 D110 D61:D79 D30:D37 D39:D48" xr:uid="{00000000-0002-0000-0000-000002000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D85:D99 D115:D1048576 D50:D58 D80:D83 D102 D109 D60:D78 D30:D37 D39:D48 D4:D6 D8:D28" xr:uid="{00000000-0002-0000-0000-000002000000}">
       <formula1>"ECE,ChemE,Phy,EE,CS,BME,BA,Others,"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E106:E1048576 E4:E104" xr:uid="{00000000-0002-0000-0000-000003000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E105:E1048576 E4:E103" xr:uid="{00000000-0002-0000-0000-000003000000}">
       <formula1>"6月,5月,7月,8月,4月,"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="B2:B64 B66:B115" xr:uid="{00000000-0002-0000-0000-000004000000}">
+    <dataValidation type="list" allowBlank="1" sqref="B65:B114 B2:B63" xr:uid="{00000000-0002-0000-0000-000004000000}">
       <formula1>"北京,上海,广州,武汉,沈阳"</formula1>
     </dataValidation>
-    <dataValidation type="list" sqref="B65" xr:uid="{00000000-0002-0000-0000-000005000000}">
+    <dataValidation type="list" sqref="B64" xr:uid="{00000000-0002-0000-0000-000005000000}">
       <formula1>"北京,上海,广州,武汉,沈阳"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="B116:B194" xr:uid="{00000000-0002-0000-0000-000006000000}">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="B115:B193" xr:uid="{00000000-0002-0000-0000-000006000000}">
       <formula1>"北京,上海,广州,武汉,沈阳"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="C2:C64 C66:C115" xr:uid="{00000000-0002-0000-0000-000007000000}">
+    <dataValidation type="list" allowBlank="1" sqref="C65:C114 C2:C63" xr:uid="{00000000-0002-0000-0000-000007000000}">
       <formula1>"PhD,Master,Bachelor"</formula1>
     </dataValidation>
-    <dataValidation type="list" sqref="C65" xr:uid="{00000000-0002-0000-0000-000008000000}">
+    <dataValidation type="list" sqref="C64" xr:uid="{00000000-0002-0000-0000-000008000000}">
       <formula1>"PhD,Master,Bachelor"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="C116:C194" xr:uid="{00000000-0002-0000-0000-000009000000}">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="C115:C193" xr:uid="{00000000-0002-0000-0000-000009000000}">
       <formula1>"PhD,Master,Bachelor"</formula1>
     </dataValidation>
-    <dataValidation type="date" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H4:H1048576 F4:F1048576" xr:uid="{00000000-0002-0000-0000-000000000000}"/>
+    <dataValidation type="date" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F4:F1048576 H4:H1048576" xr:uid="{00000000-0002-0000-0000-000000000000}"/>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G4:G1048576" xr:uid="{00000000-0002-0000-0000-000001000000}">
       <formula1>"Check,Approve,Issue,"</formula1>
     </dataValidation>

</xml_diff>